<commit_message>
apache batik lizenz hinzugefügt
</commit_message>
<xml_diff>
--- a/de.imise.tool3lgm/thirdPartyLicenses.xlsx
+++ b/de.imise.tool3lgm/thirdPartyLicenses.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="42">
   <si>
     <t>last checked</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>BSD 2-clause</t>
+  </si>
+  <si>
+    <t>org.apache.batik</t>
   </si>
 </sst>
 </file>
@@ -855,6 +858,20 @@
         <v>6</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="3">
+        <v>44113.0</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
refs #281: maven plugin hinzugefügt für die Erstellung der version.info datei + Linzenz hinzugefügt
</commit_message>
<xml_diff>
--- a/de.imise.tool3lgm/thirdPartyLicenses.xlsx
+++ b/de.imise.tool3lgm/thirdPartyLicenses.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="44">
   <si>
     <t>last checked</t>
   </si>
@@ -137,6 +137,12 @@
   </si>
   <si>
     <t>org.apache.batik</t>
+  </si>
+  <si>
+    <t>git-commit-id-maven-plugin</t>
+  </si>
+  <si>
+    <t>GNU Lesser General Public License 3.0</t>
   </si>
 </sst>
 </file>
@@ -146,7 +152,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -154,12 +160,11 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -167,7 +172,11 @@
       <color rgb="FF222222"/>
       <name val="Verdana"/>
     </font>
-    <font/>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF24292E"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -198,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -211,19 +220,16 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -613,7 +619,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6">
+      <c r="A13" s="3">
         <v>44105.0</v>
       </c>
       <c r="B13" s="2" t="s">
@@ -683,7 +689,7 @@
       <c r="B18" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="2" t="s">
@@ -747,13 +753,13 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6">
-        <v>44104.0</v>
-      </c>
-      <c r="B23" s="8" t="s">
+      <c r="A23" s="3">
+        <v>44104.0</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D23" s="2" t="s">
@@ -761,13 +767,13 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6">
-        <v>44104.0</v>
-      </c>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="3">
+        <v>44104.0</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="2" t="s">
@@ -775,13 +781,13 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6">
-        <v>44104.0</v>
-      </c>
-      <c r="B25" s="8" t="s">
+      <c r="A25" s="3">
+        <v>44104.0</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="2" t="s">
@@ -789,13 +795,13 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6">
-        <v>44104.0</v>
-      </c>
-      <c r="B26" s="8" t="s">
+      <c r="A26" s="3">
+        <v>44104.0</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D26" s="2" t="s">
@@ -803,13 +809,13 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6">
-        <v>44104.0</v>
-      </c>
-      <c r="B27" s="8" t="s">
+      <c r="A27" s="3">
+        <v>44104.0</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="2" t="s">
         <v>36</v>
       </c>
       <c r="D27" s="2" t="s">
@@ -817,13 +823,13 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6">
-        <v>44104.0</v>
-      </c>
-      <c r="B28" s="8" t="s">
+      <c r="A28" s="3">
+        <v>44104.0</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D28" s="2" t="s">
@@ -869,6 +875,20 @@
         <v>12</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3">
+        <v>44139.0</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refs #1: Git-Commit-Id-Plugin aus den Lizenzen entfernt und vorhandensein der Bibliotheken überprüft
</commit_message>
<xml_diff>
--- a/de.imise.tool3lgm/thirdPartyLicenses.xlsx
+++ b/de.imise.tool3lgm/thirdPartyLicenses.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="42">
   <si>
     <t>last checked</t>
   </si>
@@ -137,12 +137,6 @@
   </si>
   <si>
     <t>org.apache.batik</t>
-  </si>
-  <si>
-    <t>git-commit-id-maven-plugin</t>
-  </si>
-  <si>
-    <t>GNU Lesser General Public License 3.0</t>
   </si>
 </sst>
 </file>
@@ -152,7 +146,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -160,11 +154,13 @@
     </font>
     <font>
       <b/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font/>
     <font>
-      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -175,7 +171,6 @@
     <font>
       <sz val="10.0"/>
       <color rgb="FF24292E"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="4">
@@ -207,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -217,19 +212,22 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -446,6 +444,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="23.0"/>
+    <col customWidth="1" min="3" max="3" width="35.43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,7 +463,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -478,7 +477,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
@@ -492,7 +491,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
@@ -508,7 +507,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>10</v>
@@ -522,7 +521,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>11</v>
@@ -536,7 +535,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>13</v>
@@ -550,7 +549,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>14</v>
@@ -564,7 +563,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>15</v>
@@ -578,7 +577,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>16</v>
@@ -592,7 +591,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>17</v>
@@ -606,7 +605,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>18</v>
@@ -628,7 +627,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>20</v>
@@ -642,7 +641,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>21</v>
@@ -656,7 +655,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>22</v>
@@ -670,7 +669,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>23</v>
@@ -684,7 +683,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>24</v>
@@ -698,7 +697,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>26</v>
@@ -712,7 +711,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>27</v>
@@ -726,7 +725,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>28</v>
@@ -740,7 +739,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3">
-        <v>44105.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>29</v>
@@ -754,9 +753,9 @@
     </row>
     <row r="23">
       <c r="A23" s="3">
-        <v>44104.0</v>
-      </c>
-      <c r="B23" s="2" t="s">
+        <v>44172.0</v>
+      </c>
+      <c r="B23" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="6" t="s">
@@ -768,12 +767,12 @@
     </row>
     <row r="24">
       <c r="A24" s="3">
-        <v>44104.0</v>
-      </c>
-      <c r="B24" s="2" t="s">
+        <v>44172.0</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D24" s="2" t="s">
@@ -782,12 +781,12 @@
     </row>
     <row r="25">
       <c r="A25" s="3">
-        <v>44104.0</v>
-      </c>
-      <c r="B25" s="2" t="s">
+        <v>44172.0</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D25" s="2" t="s">
@@ -796,12 +795,12 @@
     </row>
     <row r="26">
       <c r="A26" s="3">
-        <v>44104.0</v>
-      </c>
-      <c r="B26" s="2" t="s">
+        <v>44172.0</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D26" s="2" t="s">
@@ -810,12 +809,12 @@
     </row>
     <row r="27">
       <c r="A27" s="3">
-        <v>44104.0</v>
-      </c>
-      <c r="B27" s="2" t="s">
+        <v>44172.0</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="7" t="s">
         <v>36</v>
       </c>
       <c r="D27" s="2" t="s">
@@ -824,12 +823,12 @@
     </row>
     <row r="28">
       <c r="A28" s="3">
-        <v>44104.0</v>
-      </c>
-      <c r="B28" s="2" t="s">
+        <v>44172.0</v>
+      </c>
+      <c r="B28" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="7" t="s">
         <v>5</v>
       </c>
       <c r="D28" s="2" t="s">
@@ -838,7 +837,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3">
-        <v>44104.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>38</v>
@@ -852,7 +851,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3">
-        <v>44105.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>39</v>
@@ -866,7 +865,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3">
-        <v>44113.0</v>
+        <v>44172.0</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>41</v>
@@ -879,18 +878,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3">
-        <v>44139.0</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A32" s="3"/>
+      <c r="C32" s="8"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
refs #421: DropDownButtonSource + pom.xml (utils) + thirdPartyLicenses.xlsx: org.netbeans.api hinzugefügt und damit die DropDownButtonSource Klasse realisiert, über die ganz einfach DropDownButtons für die Toolbar erzeugt werden können. DropdownButtons sind Buttons, mit einem kleinen Pfeil daneben, über den sich ein Dropdown-Menü öffnet, über das die Funktion des Buttons festgelegt werden kann.Damit kann man viele Funktionen in einem Button zusammenfassen.
</commit_message>
<xml_diff>
--- a/de.imise.tool3lgm/thirdPartyLicenses.xlsx
+++ b/de.imise.tool3lgm/thirdPartyLicenses.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23530"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eigene Projekte\Bitbucket\tool-3lgm2\de.imise.tool3lgm\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53428226-9CBE-43BB-A21B-F1E337A90BD5}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Tabellenblatt1" sheetId="1" r:id="rId4"/>
+    <sheet name="Tabellenblatt1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="44">
   <si>
     <t>last checked</t>
   </si>
@@ -137,40 +146,54 @@
   </si>
   <si>
     <t>org.apache.batik</t>
+  </si>
+  <si>
+    <t>org.openide</t>
+  </si>
+  <si>
+    <t>org.netbeans</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="9.0"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <color rgb="FF222222"/>
       <name val="Verdana"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF24292E"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="4">
@@ -178,7 +201,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -194,56 +217,55 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
     <border>
+      <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -433,21 +455,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="23.0"/>
-    <col customWidth="1" min="3" max="3" width="35.43"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,9 +486,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -475,9 +500,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
@@ -489,9 +514,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
@@ -505,9 +530,9 @@
       <c r="I4" s="4"/>
       <c r="J4" s="5"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>10</v>
@@ -519,9 +544,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>11</v>
@@ -533,9 +558,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>13</v>
@@ -547,9 +572,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>14</v>
@@ -561,9 +586,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>15</v>
@@ -575,9 +600,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>16</v>
@@ -589,9 +614,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>17</v>
@@ -603,9 +628,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>18</v>
@@ -617,17 +642,17 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>44105.0</v>
+        <v>44105</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>20</v>
@@ -639,9 +664,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>21</v>
@@ -653,9 +678,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>22</v>
@@ -667,9 +692,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>23</v>
@@ -681,9 +706,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>24</v>
@@ -695,9 +720,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>26</v>
@@ -709,9 +734,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>27</v>
@@ -723,9 +748,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>28</v>
@@ -737,9 +762,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>29</v>
@@ -751,9 +776,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>30</v>
@@ -765,9 +790,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>32</v>
@@ -779,9 +804,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>33</v>
@@ -793,9 +818,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>34</v>
@@ -807,9 +832,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>35</v>
@@ -821,9 +846,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>37</v>
@@ -835,9 +860,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>38</v>
@@ -849,9 +874,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>39</v>
@@ -863,9 +888,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
-        <v>44172.0</v>
+        <v>44172</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>41</v>
@@ -877,11 +902,35 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3"/>
-      <c r="C32" s="8"/>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>44227</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>44227</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Apple Start Problems
</commit_message>
<xml_diff>
--- a/de.imise.tool3lgm/thirdPartyLicenses.xlsx
+++ b/de.imise.tool3lgm/thirdPartyLicenses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eigene Projekte\Bitbucket\tool-3lgm2\de.imise.tool3lgm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\D\Eigene Projekte\Bitbucket\tool-3lgm2\de.imise.tool3lgm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53428226-9CBE-43BB-A21B-F1E337A90BD5}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D88B391A-0F2D-46DE-A77D-EFE6736A57F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabellenblatt1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="42">
   <si>
     <t>last checked</t>
   </si>
@@ -41,12 +41,6 @@
   </si>
   <si>
     <t>check</t>
-  </si>
-  <si>
-    <t>AppleJavaExtensions</t>
-  </si>
-  <si>
-    <t>apple license</t>
   </si>
   <si>
     <t>checker-qual</t>
@@ -465,14 +459,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="35.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -486,7 +480,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>44172</v>
       </c>
@@ -500,7 +494,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>44172</v>
       </c>
@@ -508,18 +502,20 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="5"/>
+    </row>
+    <row r="4" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>5</v>
@@ -527,24 +523,22 @@
       <c r="D4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>44172</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>44172</v>
       </c>
@@ -552,287 +546,287 @@
         <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>44105</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>44105</v>
-      </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="D17" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>44172</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="D22" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>44172</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B24" s="7" t="s">
+      <c r="C24" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B25" s="7" t="s">
+      <c r="C25" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B26" s="7" t="s">
+      <c r="C26" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>12</v>
-      </c>
       <c r="D26" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>44172</v>
       </c>
@@ -840,41 +834,41 @@
         <v>35</v>
       </c>
       <c r="C27" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B28" s="7" t="s">
+      <c r="C28" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>44172</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="D29" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>44172</v>
       </c>
@@ -882,51 +876,37 @@
         <v>39</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>44227</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="3">
-        <v>44172</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>12</v>
+      <c r="C31" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>44227</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="3">
-        <v>44227</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" s="2" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>